<commit_message>
Match Merit lookup keys to original source text
</commit_message>
<xml_diff>
--- a/downloads/Merit_2026_Employee_Bulk_Calculator_350_exact.xlsx
+++ b/downloads/Merit_2026_Employee_Bulk_Calculator_350_exact.xlsx
@@ -22729,7 +22729,7 @@
     <row r="114">
       <c r="A114" s="92" t="inlineStr">
         <is>
-          <t>CQ engineer Site Engineering P1-G midpoint (CQ=Commissioning&amp;Qualification)</t>
+          <t xml:space="preserve">CQ engineer  Site Engineering P1-G midpoint   (CQ=Commissioning&amp;Qualification)</t>
         </is>
       </c>
       <c r="B114" s="92" t="inlineStr">
@@ -22746,7 +22746,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>CQ engineer Site Engineering P1-F midpoint (CQ=Commissioning&amp;Qualification)</t>
+          <t xml:space="preserve">CQ engineer Site Engineering P1-F midpoint   (CQ=Commissioning&amp;Qualification)</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -22763,7 +22763,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>CQ engineer Site Engineering P1-G Tussen midpoint en max. (CQ=Commissioning&amp;Qualification)</t>
+          <t xml:space="preserve">CQ engineer Site Engineering P1-G Tussen midpoint en max.   (CQ=Commissioning&amp;Qualification)</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -22780,7 +22780,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>SPOC=Programma-manager Site Engineering P3-J Tussen midpoint en max.</t>
+          <t xml:space="preserve">SPOC=Programma-manager Site Engineering  P3-J  Tussen midpoint en max.</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">

</xml_diff>